<commit_message>
Improve Researchr deadline scraping
</commit_message>
<xml_diff>
--- a/deadline.xlsx
+++ b/deadline.xlsx
@@ -534,17 +534,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>52</t>
+          <t>1037</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ACM International Conference on the Foundations of Software Engineering (was ESEC/FSE, changed 2024; duplicate previously listed as ESEC, removed from DB)</t>
+          <t>International Conference on Functional Programming</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>FSE</t>
+          <t>ICFP</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -554,7 +554,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>A*</t>
+          <t>A</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -569,29 +569,45 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>https://www.myhuiban.com/conference/87?page=1</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
+          <t>https://conf.researchr.org/dates/icfp-2026</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>14 May 2026</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>15 Jun 2026</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>4 days 9 hours</t>
+        </is>
+      </c>
       <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>1412</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ACM International Symposium on Computer Architecture</t>
+          <t>International Symposium on Software Testing and Analysis</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ISCA</t>
+          <t>ISSTA</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -601,7 +617,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>A*</t>
+          <t>A</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -611,40 +627,54 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>CSE</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>4606</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>4612</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
+          <t>4612</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/dates/issta-2026</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>15 Jun 2026</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>4 Aug 2026</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>4 days 9 hours</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>not exceed 2 pages; double-column</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>676</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ACM-SIGACT Symposium on Principles of Programming Languages</t>
+          <t>IEEE International Conference on Software Maintenance and Evolution (prior to 2014 was ICSM, IEEE International Conference on Software Maintenance)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>POPL</t>
+          <t>ICSME</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -654,7 +684,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>A*</t>
+          <t>A</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -667,27 +697,47 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/icsme-2026</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>18 Jun 2026</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>4 Jun 2026</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>7 days 9 hours</t>
+        </is>
+      </c>
       <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>2165</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ACM-SIGPLAN Conference on Programming Language Design and Implementation</t>
+          <t>European Conference on Software Architecture</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>PLDI</t>
+          <t>ECSA</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -697,7 +747,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>A*</t>
+          <t>B</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -710,27 +760,47 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/dates/ecsa-2026</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>1 May 2026</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>29 Jun 2026</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>18 days 9 hours</t>
+        </is>
+      </c>
       <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>147</t>
+          <t>279</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Architectural Support for Programming Languages and Operating Systems</t>
+          <t>Automated Software Engineering Conference</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ASPLOS</t>
+          <t>ASE</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -753,32 +823,51 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>4606</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/dates/ase-2026</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>10 Jul 2026</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>21 Aug 2026</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>29 days 9 hours</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>4-8 pages</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>279</t>
+          <t>1244</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Automated Software Engineering Conference</t>
+          <t>International Conference on Model Driven Engineering Languages and Systems (Previously UML, changed in 2005)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ASE</t>
+          <t>MODELS</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -788,7 +877,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>A*</t>
+          <t>A</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -801,27 +890,47 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/dates/models-2026</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>10 Jul 2026</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>26 Aug 2026</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>29 days 9 hours</t>
+        </is>
+      </c>
       <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>331</t>
+          <t>171</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Computer Aided Verification</t>
+          <t>ASIAN Symposium on Programming Languages and Systems</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>CAV</t>
+          <t>APLAS</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -831,7 +940,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>A*</t>
+          <t>B</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -844,32 +953,51 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>4613</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/track/aplas-atva-2026/aplas-2026</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>26 Sep 2026</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>24 Jul 2026</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>43 days 9 hours</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>not exceed 17 pages; LNCS format</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1209</t>
+          <t>1696</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>International Conference on Software Engineering</t>
+          <t>Product Focused Software Process Improvement</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ICSE</t>
+          <t>PROFES</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -879,7 +1007,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>A*</t>
+          <t>B</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -892,27 +1020,47 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/track/profes-2026/profes-2026-short-papers-and-posters</t>
+        </is>
+      </c>
       <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>11 Sep 2026</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>92 days 9 hours</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>8 pages; LNCS format</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>711</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Measurement and Modeling of Computer Systems</t>
+          <t>IEEE International Working Conference on Mining Software Repositories</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>SIGMETRICS</t>
+          <t>MSR</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -922,7 +1070,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>A*</t>
+          <t>A</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -935,27 +1083,48 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>4605</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/msr-2026</t>
+        </is>
+      </c>
       <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>28 Sep 2026</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>109 days 9 hours</t>
+        </is>
+      </c>
       <c r="O10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>791</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ACM Conference on Object Oriented Programming Systems Languages and Applications</t>
+          <t>International Conference on Software Architecture (was previously WICSA)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>OOPSLA</t>
+          <t>ICSA</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -978,27 +1147,47 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/dates/icsa-2027</t>
+        </is>
+      </c>
       <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>19 Jan 2027</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>2027-01-19</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>222 days 9 hours</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>maximum of 8 pages; IEEE format</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>421</t>
+          <t>1209</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Design, Automation and Test in Europe Conference</t>
+          <t>International Conference on Software Engineering</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>DATE</t>
+          <t>ICSE</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1008,7 +1197,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>A*</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1018,35 +1207,50 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>CSE</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>4612</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
+          <t>4612</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/dates/icse-2027</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>27 Jan 2027</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>29 Jan 2027</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>2027-01-27</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>230 days 9 hours</t>
+        </is>
+      </c>
       <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>488</t>
+          <t>1221</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>European Conference on Object-Oriented Programming</t>
+          <t>International Conference on Software Testing, Verification and Validation</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ECOOP</t>
+          <t>ICST</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1069,27 +1273,43 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/icst-2027</t>
+        </is>
+      </c>
       <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>20 Feb 2027</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>2027-02-20</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>254 days 9 hours</t>
+        </is>
+      </c>
       <c r="O13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>514</t>
+          <t>1521</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>European Symposium on Programming</t>
+          <t>International Workshop on Requirements Engineering: Foundation for Software Quality</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ESOP</t>
+          <t>REFSQ</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1099,7 +1319,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1112,27 +1332,47 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/refsq-2027</t>
+        </is>
+      </c>
       <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>11 Mar 2027</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>2027-03-11</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>273 days 9 hours</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>4 pages</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1181</t>
+          <t>52</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>IEEE International Conference on Program Comprehension (previously IWPC, changed in 2006)</t>
+          <t>ACM International Conference on the Foundations of Software Engineering (was ESEC/FSE, changed 2024; duplicate previously listed as ESEC, removed from DB)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ICPC</t>
+          <t>FSE</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1142,7 +1382,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>A*</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1155,27 +1395,47 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/fse-2027</t>
+        </is>
+      </c>
       <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>31 Mar 2027</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>2027-03-31</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>293 days 9 hours</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>no more than 18 pages; single-column</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2280</t>
+          <t>1763</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>IEEE International Conference on Software Analysis, Evolution and Reengineering</t>
+          <t>Static Analysis Symposium</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>SANER</t>
+          <t>SAS</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1185,7 +1445,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1198,27 +1458,47 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr"/>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/sas-2026</t>
+        </is>
+      </c>
       <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
-      <c r="O16" t="inlineStr"/>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>1 May 2026</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>overdue by 40 days 14 hours</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>LNCS format</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>676</t>
+          <t>1215</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>IEEE International Conference on Software Maintenance and Evolution (prior to 2014 was ICSM, IEEE International Conference on Software Maintenance)</t>
+          <t>International Conference on Software Language Engineering</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ICSME</t>
+          <t>SLE</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1228,7 +1508,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1241,27 +1521,47 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr"/>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/sle-2026</t>
+        </is>
+      </c>
       <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
-      <c r="O17" t="inlineStr"/>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>20 Apr 2026</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>overdue by 51 days 14 hours</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>6-12 pages</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>690</t>
+          <t>2283</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>IEEE International Requirements Engineering Conference</t>
+          <t>International Symposium on Search Based Software Engineering</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>RE</t>
+          <t>SSBSE</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1271,7 +1571,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1284,27 +1584,52 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>4602</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/track/ssbse-2026/ssbse-2026-ssbse-challenge</t>
+        </is>
+      </c>
       <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>9 Apr 2026</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>overdue by 62 days 14 hours</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>LNCS format</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>711</t>
+          <t>84</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>IEEE International Working Conference on Mining Software Repositories</t>
+          <t>ACM-SIGPLAN Conference on Programming Language Design and Implementation</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>MSR</t>
+          <t>PLDI</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1314,7 +1639,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>A*</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1327,32 +1652,51 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>4605</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/dates/pldi-2026</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>17 Mar 2026</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>4 May 2026</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>overdue by 85 days 14 hours</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>26 pages</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>878</t>
+          <t>690</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>International Conference in Business Process Management</t>
+          <t>IEEE International Requirements Engineering Conference</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>BPM</t>
+          <t>RE</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1367,7 +1711,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1375,27 +1719,47 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/dates/RE-2026</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>13 Mar 2026</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>22 May 2026</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>overdue by 89 days 14 hours</t>
+        </is>
+      </c>
       <c r="O20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1022</t>
+          <t>1376</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>International Conference on Evaluation and Assessment in Software Engineering</t>
+          <t>International Symposium on Empirical Software Engineering and Measurement</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>EASE</t>
+          <t>ESEM</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1418,27 +1782,47 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr"/>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/esem-2026</t>
+        </is>
+      </c>
       <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr"/>
-      <c r="O21" t="inlineStr"/>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>13 Mar 2026</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>overdue by 89 days 14 hours</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>LIPIcs format</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1037</t>
+          <t>1039</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>International Conference on Functional Programming</t>
+          <t>International Conference on Generative Programming and Component Engineering</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ICFP</t>
+          <t>GPCE</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1448,12 +1832,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1461,27 +1845,47 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr"/>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/gpce-2026</t>
+        </is>
+      </c>
       <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr"/>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>12 Mar 2026</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>2026-03-12</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>overdue by 90 days 14 hours</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>not exceed 10 pages</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>1244</t>
+          <t>488</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>International Conference on Model Driven Engineering Languages and Systems (Previously UML, changed in 2005)</t>
+          <t>European Conference on Object-Oriented Programming</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>MODELS</t>
+          <t>ECOOP</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1504,27 +1908,47 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/dates/ecoop-2026</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>8 May 2026</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>24 Feb 2026</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>overdue by 106 days 14 hours</t>
+        </is>
+      </c>
       <c r="O23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>791</t>
+          <t>1022</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>International Conference on Software Architecture (was previously WICSA)</t>
+          <t>International Conference on Evaluation and Assessment in Software Engineering</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ICSA</t>
+          <t>EASE</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1547,27 +1971,47 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/dates/ease-2026</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>23 Feb 2026</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>30 Apr 2026</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>overdue by 107 days 14 hours</t>
+        </is>
+      </c>
       <c r="O24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>1221</t>
+          <t>355</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>International Conference on Software Testing, Verification and Validation</t>
+          <t>Conference on Agile Software Development</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ICST</t>
+          <t>XP</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1577,7 +2021,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1590,27 +2034,43 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr"/>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/dates/xp-2026</t>
+        </is>
+      </c>
       <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>20 Feb 2026</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>overdue by 110 days 14 hours</t>
+        </is>
+      </c>
       <c r="O25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>1314</t>
+          <t>2287</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>International Joint Conference on Automated Reasoning</t>
+          <t>European Conference on Modelling Foundations and Applications</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>IJCAR</t>
+          <t>ECMFA</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1620,7 +2080,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1630,40 +2090,54 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>4602</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>4612</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>4613</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
+          <t>4612</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/ecmfa-2026</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>6 Feb 2026</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>13 Feb 2026</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>overdue by 124 days 14 hours</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>not exceed 14 pages</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>1362</t>
+          <t>2348</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>International Symposium on Code Generation and Optimization</t>
+          <t>International Conference on Cooperative and Human Aspects of Software Engineering</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>CGO</t>
+          <t>CHASE</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1673,40 +2147,61 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>4612</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr"/>
+          <t>4608</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>4612</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/track/chase-2026/chase-2026-voices-of-the-industry-track</t>
+        </is>
+      </c>
       <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>February 2nd, 2026</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>overdue by 128 days 14 hours</t>
+        </is>
+      </c>
       <c r="O27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>1376</t>
+          <t>2288</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>International Symposium on Empirical Software Engineering and Measurement</t>
+          <t>International Conference on Technical Debt</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>ESEM</t>
+          <t>TechDebt</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1716,7 +2211,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1729,27 +2224,43 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr"/>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/dates/techdebt-2026</t>
+        </is>
+      </c>
       <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>22 Jan 2026</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>overdue by 139 days 14 hours</t>
+        </is>
+      </c>
       <c r="O28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2281</t>
+          <t>1847</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>International Symposium on Software Engineering for Adaptive and Self-Managing Systems</t>
+          <t>Verification, Model Checking and Abstract Interpretation</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>SEAMS</t>
+          <t>VMCAI</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1759,12 +2270,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1772,27 +2283,47 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/details/VMCAI-2026/VMCAI-2026-papers/2/TypedC-Spatial-Memory-Safety-for-Low-Level-Programs-by-Abstract-Interpretation</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>13 Jan 2026</t>
+        </is>
+      </c>
       <c r="L29" t="inlineStr"/>
-      <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
-      <c r="O29" t="inlineStr"/>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>overdue by 148 days 14 hours</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>20 pages; LNCS format</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>1411</t>
+          <t>1181</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>International Symposium on Software Reliability Engineering</t>
+          <t>IEEE International Conference on Program Comprehension (previously IWPC, changed in 2006)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>ISSRE</t>
+          <t>ICPC</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1815,27 +2346,43 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr"/>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/dates/icpc-2026</t>
+        </is>
+      </c>
       <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
-      <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr"/>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>12 Jan 2026</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>overdue by 149 days 14 hours</t>
+        </is>
+      </c>
       <c r="O30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>1412</t>
+          <t>540</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>International Symposium on Software Testing and Analysis</t>
+          <t>International Symposium on Formal Methods (was Formal Methods Europe FME)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>ISSTA</t>
+          <t>FM</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1845,7 +2392,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1858,27 +2405,52 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>4613</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/dates/fm-2026</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>6 Feb 2026</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>9 Jan 2026</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>2026-01-09</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>overdue by 152 days 14 hours</t>
+        </is>
+      </c>
       <c r="O31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>1818</t>
+          <t>2281</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Tools and Algorithms for Construction and Analysis of Systems</t>
+          <t>International Symposium on Software Engineering for Adaptive and Self-Managing Systems</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>TACAS</t>
+          <t>SEAMS</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1901,27 +2473,47 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr"/>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/track/seams-2026/seams-2026-research-track</t>
+        </is>
+      </c>
       <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr"/>
-      <c r="O32" t="inlineStr"/>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>5th January 2026</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>2026-01-05</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>overdue by 156 days 14 hours</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>10 pages of content; ACM format</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2278</t>
+          <t>32</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>ACM/SPEC International Conference on Performance Engineering</t>
+          <t>ACM International Symposium on Computer Architecture</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ICPE</t>
+          <t>ISCA</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1931,7 +2523,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A*</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1941,7 +2533,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>4612</t>
+          <t>CSE</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -1949,7 +2541,16 @@
           <t>4606</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr"/>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>4612</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/isca-2027</t>
+        </is>
+      </c>
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr"/>
@@ -1959,17 +2560,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>171</t>
+          <t>82</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>ASIAN Symposium on Programming Languages and Systems</t>
+          <t>ACM-SIGACT Symposium on Principles of Programming Languages</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>APLAS</t>
+          <t>POPL</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1979,7 +2580,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A*</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1992,7 +2593,11 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr"/>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/popl-2027</t>
+        </is>
+      </c>
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr"/>
@@ -2002,17 +2607,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2341</t>
+          <t>147</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Certified Programs and Proofs</t>
+          <t>Architectural Support for Programming Languages and Operating Systems</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>CPP</t>
+          <t>ASPLOS</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -2022,7 +2627,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A*</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2032,15 +2637,19 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>4613</t>
+          <t>4612</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>4612</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr"/>
+          <t>4606</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/asplos-2027</t>
+        </is>
+      </c>
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
@@ -2050,17 +2659,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>355</t>
+          <t>331</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Conference on Agile Software Development</t>
+          <t>Computer Aided Verification</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>XP</t>
+          <t>CAV</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2070,7 +2679,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A*</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2083,7 +2692,16 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr"/>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>4613</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/cav-2027</t>
+        </is>
+      </c>
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
@@ -2093,17 +2711,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>464</t>
+          <t>39</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Euromicro Conference on Software Engineering and Advanced Applications</t>
+          <t>Measurement and Modeling of Computer Systems</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>SEAA</t>
+          <t>SIGMETRICS</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2113,12 +2731,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A*</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2126,12 +2744,11 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>4601</t>
-        </is>
-      </c>
-      <c r="J37" t="inlineStr"/>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/sigmetrics-2027</t>
+        </is>
+      </c>
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr"/>
@@ -2141,17 +2758,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2287</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>European Conference on Modelling Foundations and Applications</t>
+          <t>ACM Conference on Object Oriented Programming Systems Languages and Applications</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ECMFA</t>
+          <t>OOPSLA</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2161,7 +2778,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2174,7 +2791,11 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr"/>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/oopsla-2027</t>
+        </is>
+      </c>
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
@@ -2184,17 +2805,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2165</t>
+          <t>421</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>European Conference on Software Architecture</t>
+          <t>Design, Automation and Test in Europe Conference</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ECSA</t>
+          <t>DATE</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2204,7 +2825,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2214,10 +2835,19 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>4612</t>
-        </is>
-      </c>
-      <c r="J39" t="inlineStr"/>
+          <t>CSE</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>4612</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/date-2027</t>
+        </is>
+      </c>
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
@@ -2227,17 +2857,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>510</t>
+          <t>514</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>European SPI</t>
+          <t>European Symposium on Programming</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>EuroSPI</t>
+          <t>ESOP</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2247,7 +2877,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2260,7 +2890,11 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr"/>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/esop-2027</t>
+        </is>
+      </c>
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr"/>
@@ -2270,17 +2904,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2196</t>
+          <t>2280</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Formal Methods in Computer-Aided Design</t>
+          <t>IEEE International Conference on Software Analysis, Evolution and Reengineering</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>FMCAD</t>
+          <t>SANER</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2290,7 +2924,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2303,27 +2937,35 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr"/>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/saner-2027</t>
+        </is>
+      </c>
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr"/>
       <c r="N41" t="inlineStr"/>
-      <c r="O41" t="inlineStr"/>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>not exceed 10 pages</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>547</t>
+          <t>878</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Foundations of Software Science and Computational Structures</t>
+          <t>International Conference in Business Process Management</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>FOSSACS</t>
+          <t>BPM</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2333,25 +2975,24 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>4613</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>4612</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr"/>
+          <t>4612</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/bpm-2027</t>
+        </is>
+      </c>
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr"/>
@@ -2361,17 +3002,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>554</t>
+          <t>1314</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Fundamental Approaches to Software Engineering</t>
+          <t>International Joint Conference on Automated Reasoning</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>FASE</t>
+          <t>IJCAR</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -2381,7 +3022,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2391,10 +3032,24 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>4612</t>
-        </is>
-      </c>
-      <c r="J43" t="inlineStr"/>
+          <t>4602</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>4612</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>4613</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/ijcar-2027</t>
+        </is>
+      </c>
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr"/>
@@ -2404,17 +3059,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>648</t>
+          <t>1362</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>IEEE International Conference on e-Science and Grid Computing</t>
+          <t>International Symposium on Code Generation and Optimization</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>e-Science</t>
+          <t>CGO</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -2424,50 +3079,48 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>4606</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>4601</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>4612</t>
-        </is>
-      </c>
-      <c r="J44" t="inlineStr"/>
+          <t>4612</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/cgo-2027</t>
+        </is>
+      </c>
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr"/>
       <c r="M44" t="inlineStr"/>
       <c r="N44" t="inlineStr"/>
-      <c r="O44" t="inlineStr"/>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>up to 11 pages; ACM format</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>646</t>
+          <t>1411</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>IEEE International Conference on Engineering of Complex Computer Systems</t>
+          <t>International Symposium on Software Reliability Engineering</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>ICECCS</t>
+          <t>ISSRE</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -2477,7 +3130,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2490,12 +3143,11 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>4606</t>
-        </is>
-      </c>
-      <c r="J45" t="inlineStr"/>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/issre-2027</t>
+        </is>
+      </c>
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr"/>
       <c r="M45" t="inlineStr"/>
@@ -2505,17 +3157,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>705</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>IEEE International Symposium on Performance Analysis of Systems and Software</t>
+          <t>Tools and Algorithms for Construction and Analysis of Systems</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>ISPASS</t>
+          <t>TACAS</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2525,7 +3177,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2538,7 +3190,11 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr"/>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/tacas-2027</t>
+        </is>
+      </c>
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr"/>
       <c r="M46" t="inlineStr"/>
@@ -2548,17 +3204,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>720</t>
+          <t>2278</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>IEEE International Working Conference on Software Visualisation</t>
+          <t>ACM/SPEC International Conference on Performance Engineering</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>VISSOFT</t>
+          <t>ICPE</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2573,20 +3229,24 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>4608</t>
+          <t>4612</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>4612</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr"/>
+          <t>4606</t>
+        </is>
+      </c>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/icpe-2027</t>
+        </is>
+      </c>
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr"/>
       <c r="M47" t="inlineStr"/>
@@ -2596,17 +3256,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>842</t>
+          <t>2341</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Integrated Formal Methods</t>
+          <t>Certified Programs and Proofs</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>IFM</t>
+          <t>CPP</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2626,15 +3286,19 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>4612</t>
+          <t>4613</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>4613</t>
-        </is>
-      </c>
-      <c r="J48" t="inlineStr"/>
+          <t>4612</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/cpp-2027</t>
+        </is>
+      </c>
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr"/>
       <c r="M48" t="inlineStr"/>
@@ -2644,17 +3308,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2337</t>
+          <t>464</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>International Conference on AI Engineering – Software Engineering for AI</t>
+          <t>Euromicro Conference on Software Engineering and Advanced Applications</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>CAIN</t>
+          <t>SEAA</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -2669,7 +3333,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -2679,10 +3343,14 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>4602</t>
-        </is>
-      </c>
-      <c r="J49" t="inlineStr"/>
+          <t>4601</t>
+        </is>
+      </c>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/seaa-2027</t>
+        </is>
+      </c>
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr"/>
       <c r="M49" t="inlineStr"/>
@@ -2692,17 +3360,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2348</t>
+          <t>510</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>International Conference on Cooperative and Human Aspects of Software Engineering</t>
+          <t>European SPI</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>CHASE</t>
+          <t>EuroSPI</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -2722,15 +3390,14 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>4608</t>
-        </is>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>4612</t>
-        </is>
-      </c>
-      <c r="J50" t="inlineStr"/>
+          <t>4612</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/eurospi-2027</t>
+        </is>
+      </c>
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr"/>
       <c r="M50" t="inlineStr"/>
@@ -2740,17 +3407,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>1023</t>
+          <t>2196</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>International Conference on Evaluation of Novel Approaches to Software Engineering</t>
+          <t>Formal Methods in Computer-Aided Design</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>ENASE</t>
+          <t>FMCAD</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -2773,7 +3440,11 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr"/>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/fmcad-2027</t>
+        </is>
+      </c>
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr"/>
       <c r="M51" t="inlineStr"/>
@@ -2783,17 +3454,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>1039</t>
+          <t>547</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>International Conference on Generative Programming and Component Engineering</t>
+          <t>Foundations of Software Science and Computational Structures</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>GPCE</t>
+          <t>FOSSACS</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2808,15 +3479,24 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>4612</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr"/>
+          <t>4613</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>4612</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/fossacs-2027</t>
+        </is>
+      </c>
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr"/>
       <c r="M52" t="inlineStr"/>
@@ -2826,17 +3506,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>1119</t>
+          <t>554</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>International Conference on Logic Programming</t>
+          <t>Fundamental Approaches to Software Engineering</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>ICLP</t>
+          <t>FASE</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -2856,15 +3536,14 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>4613</t>
-        </is>
-      </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>4612</t>
-        </is>
-      </c>
-      <c r="J53" t="inlineStr"/>
+          <t>4612</t>
+        </is>
+      </c>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/fase-2027</t>
+        </is>
+      </c>
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr"/>
       <c r="M53" t="inlineStr"/>
@@ -2874,17 +3553,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2245</t>
+          <t>648</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>International Conference on Network Softwarization</t>
+          <t>IEEE International Conference on e-Science and Grid Computing</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>NetSoft</t>
+          <t>e-Science</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -2909,10 +3588,19 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>4612</t>
-        </is>
-      </c>
-      <c r="J54" t="inlineStr"/>
+          <t>4601</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>4612</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/e-science-2027</t>
+        </is>
+      </c>
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr"/>
       <c r="M54" t="inlineStr"/>
@@ -2922,17 +3610,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>1932</t>
+          <t>646</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>International Conference on Runtime Verification (was workshop pre 2010)</t>
+          <t>IEEE International Conference on Engineering of Complex Computer Systems</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>RV</t>
+          <t>ICECCS</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -2955,7 +3643,16 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="J55" t="inlineStr"/>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>4606</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/iceccs-2027</t>
+        </is>
+      </c>
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr"/>
       <c r="M55" t="inlineStr"/>
@@ -2965,17 +3662,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>1217</t>
+          <t>705</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>International Conference on Software and System Processes (was ICSP prior to 2011)</t>
+          <t>IEEE International Symposium on Performance Analysis of Systems and Software</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>ICSSP</t>
+          <t>ISPASS</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -2998,7 +3695,11 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr"/>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/ispass-2027</t>
+        </is>
+      </c>
       <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr"/>
       <c r="M56" t="inlineStr"/>
@@ -3008,17 +3709,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>1211</t>
+          <t>720</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>International Conference on Software Engineering and Formal Methods</t>
+          <t>IEEE International Working Conference on Software Visualisation</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>SEFM</t>
+          <t>VISSOFT</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -3033,15 +3734,24 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>4612</t>
-        </is>
-      </c>
-      <c r="J57" t="inlineStr"/>
+          <t>4608</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>4612</t>
+        </is>
+      </c>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/vissoft-2027</t>
+        </is>
+      </c>
       <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr"/>
       <c r="M57" t="inlineStr"/>
@@ -3051,17 +3761,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>1215</t>
+          <t>842</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>International Conference on Software Language Engineering</t>
+          <t>Integrated Formal Methods</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>SLE</t>
+          <t>IFM</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -3084,7 +3794,16 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="J58" t="inlineStr"/>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>4613</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/ifm-2027</t>
+        </is>
+      </c>
       <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr"/>
       <c r="M58" t="inlineStr"/>
@@ -3094,17 +3813,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>1220</t>
+          <t>2337</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>International Conference on Software Reuse</t>
+          <t>International Conference on AI Engineering – Software Engineering for AI</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>ICSR</t>
+          <t>CAIN</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -3127,7 +3846,16 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="J59" t="inlineStr"/>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>4602</t>
+        </is>
+      </c>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/cain-2027</t>
+        </is>
+      </c>
       <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr"/>
       <c r="M59" t="inlineStr"/>
@@ -3137,17 +3865,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2288</t>
+          <t>1023</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>International Conference on Technical Debt</t>
+          <t>International Conference on Evaluation of Novel Approaches to Software Engineering</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>TechDebt</t>
+          <t>ENASE</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -3170,7 +3898,11 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="J60" t="inlineStr"/>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/enase-2027</t>
+        </is>
+      </c>
       <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr"/>
       <c r="M60" t="inlineStr"/>
@@ -3180,17 +3912,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>1357</t>
+          <t>1119</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>International Symposium on Automated Technology for Verification and Analysis</t>
+          <t>International Conference on Logic Programming</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>ATVA</t>
+          <t>ICLP</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -3210,10 +3942,19 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>4612</t>
-        </is>
-      </c>
-      <c r="J61" t="inlineStr"/>
+          <t>4613</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>4612</t>
+        </is>
+      </c>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/iclp-2027</t>
+        </is>
+      </c>
       <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr"/>
       <c r="M61" t="inlineStr"/>
@@ -3223,17 +3964,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>540</t>
+          <t>2245</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>International Symposium on Formal Methods (was Formal Methods Europe FME)</t>
+          <t>International Conference on Network Softwarization</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>FM</t>
+          <t>NetSoft</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -3253,15 +3994,19 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>4612</t>
+          <t>4606</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>4613</t>
-        </is>
-      </c>
-      <c r="J62" t="inlineStr"/>
+          <t>4612</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/netsoft-2027</t>
+        </is>
+      </c>
       <c r="K62" t="inlineStr"/>
       <c r="L62" t="inlineStr"/>
       <c r="M62" t="inlineStr"/>
@@ -3271,17 +4016,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2283</t>
+          <t>1932</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>International Symposium on Search Based Software Engineering</t>
+          <t>International Conference on Runtime Verification (was workshop pre 2010)</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>SSBSE</t>
+          <t>RV</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -3304,12 +4049,11 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>4602</t>
-        </is>
-      </c>
-      <c r="J63" t="inlineStr"/>
+      <c r="J63" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/rv-2027</t>
+        </is>
+      </c>
       <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr"/>
       <c r="M63" t="inlineStr"/>
@@ -3319,17 +4063,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>1521</t>
+          <t>1217</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>International Workshop on Requirements Engineering: Foundation for Software Quality</t>
+          <t>International Conference on Software and System Processes (was ICSP prior to 2011)</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>REFSQ</t>
+          <t>ICSSP</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -3352,7 +4096,11 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="J64" t="inlineStr"/>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/icssp-2027</t>
+        </is>
+      </c>
       <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr"/>
       <c r="M64" t="inlineStr"/>
@@ -3362,17 +4110,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>1696</t>
+          <t>1211</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Product Focused Software Process Improvement</t>
+          <t>International Conference on Software Engineering and Formal Methods</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>PROFES</t>
+          <t>SEFM</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -3395,7 +4143,11 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="J65" t="inlineStr"/>
+      <c r="J65" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/sefm-2027</t>
+        </is>
+      </c>
       <c r="K65" t="inlineStr"/>
       <c r="L65" t="inlineStr"/>
       <c r="M65" t="inlineStr"/>
@@ -3405,17 +4157,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2282</t>
+          <t>1220</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Software Product Lines Conference</t>
+          <t>International Conference on Software Reuse</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>SPLC</t>
+          <t>ICSR</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -3438,17 +4190,11 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="H66" t="inlineStr">
-        <is>
-          <t>4601</t>
-        </is>
-      </c>
-      <c r="I66" t="inlineStr">
-        <is>
-          <t>4602</t>
-        </is>
-      </c>
-      <c r="J66" t="inlineStr"/>
+      <c r="J66" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/icsr-2027</t>
+        </is>
+      </c>
       <c r="K66" t="inlineStr"/>
       <c r="L66" t="inlineStr"/>
       <c r="M66" t="inlineStr"/>
@@ -3458,17 +4204,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>1763</t>
+          <t>1357</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Static Analysis Symposium</t>
+          <t>International Symposium on Automated Technology for Verification and Analysis</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>SAS</t>
+          <t>ATVA</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -3491,7 +4237,11 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="J67" t="inlineStr"/>
+      <c r="J67" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/atva-2027</t>
+        </is>
+      </c>
       <c r="K67" t="inlineStr"/>
       <c r="L67" t="inlineStr"/>
       <c r="M67" t="inlineStr"/>
@@ -3501,17 +4251,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>1847</t>
+          <t>2282</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Verification, Model Checking and Abstract Interpretation</t>
+          <t>Software Product Lines Conference</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>VMCAI</t>
+          <t>SPLC</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -3526,7 +4276,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -3534,7 +4284,21 @@
           <t>4612</t>
         </is>
       </c>
-      <c r="J68" t="inlineStr"/>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>4601</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>4602</t>
+        </is>
+      </c>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/splc-2027</t>
+        </is>
+      </c>
       <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr"/>
       <c r="M68" t="inlineStr"/>
@@ -6255,6 +7019,72 @@
   <autoFilter ref="A1:O133"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J57" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J58" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J59" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J60" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J61" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J62" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J63" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J64" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J65" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J66" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J67" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J68" r:id="rId67"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>